<commit_message>
Enhance PDF and Excel reports with professional branding and layout
Refactor `exportReportPdf` and `exportReportExcel` to incorporate brand colors (navy and gold), a card-based KPI layout, and improved table styling for a more polished client-facing document.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 0e10bf15-1a2d-43bc-934e-464c51d00f66
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: e2eec50e-a8a8-4f78-8545-ad32e9db4013
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/9f621e76-a1cb-47c9-a804-6aa67d168f25/0e10bf15-1a2d-43bc-934e-464c51d00f66/XeAym1z
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/exports/kpi-report-sample.xlsx
+++ b/exports/kpi-report-sample.xlsx
@@ -37,7 +37,7 @@
     <t>Report generated</t>
   </si>
   <si>
-    <t>21 July 2026, 21:10</t>
+    <t>22 July 2026, 08:45</t>
   </si>
   <si>
     <t>OPERATIONAL</t>
@@ -165,12 +165,12 @@
     </font>
     <font>
       <b/>
-      <color rgb="FF1E3A5F"/>
+      <color rgb="FF1B2A4A"/>
       <sz val="14"/>
     </font>
     <font>
       <b/>
-      <color rgb="FF1E3A5F"/>
+      <color rgb="FF1B2A4A"/>
     </font>
     <font>
       <b/>
@@ -186,16 +186,16 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF1E3A5F"/>
+        <fgColor rgb="FF1B2A4A"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFEBEFF5"/>
+        <fgColor rgb="FFF4F6FA"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -203,16 +203,26 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FFBF9854"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -607,13 +617,14 @@
     <col min="2" max="2" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>0</v>
       </c>
+      <c r="B5" s="2"/>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" s="2" t="s">
+      <c r="A6" s="3" t="s">
         <v>1</v>
       </c>
       <c r="B6" t="s">
@@ -621,7 +632,7 @@
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" s="2" t="s">
+      <c r="A7" s="3" t="s">
         <v>3</v>
       </c>
       <c r="B7" t="s">
@@ -629,7 +640,7 @@
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A8" s="2" t="s">
+      <c r="A8" s="3" t="s">
         <v>5</v>
       </c>
       <c r="B8" t="s">
@@ -637,7 +648,7 @@
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A9" s="2" t="s">
+      <c r="A9" s="3" t="s">
         <v>7</v>
       </c>
       <c r="B9" t="s">
@@ -645,16 +656,16 @@
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A11" s="3" t="s">
+      <c r="A11" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="B11" s="4"/>
+      <c r="B11" s="5"/>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A12" s="5" t="s">
+      <c r="A12" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="B12" s="5" t="s">
+      <c r="B12" s="6" t="s">
         <v>11</v>
       </c>
     </row>
@@ -662,7 +673,7 @@
       <c r="A13" t="s">
         <v>12</v>
       </c>
-      <c r="B13" s="6" t="s">
+      <c r="B13" s="7" t="s">
         <v>13</v>
       </c>
     </row>
@@ -670,7 +681,7 @@
       <c r="A14" t="s">
         <v>14</v>
       </c>
-      <c r="B14" s="6" t="s">
+      <c r="B14" s="7" t="s">
         <v>15</v>
       </c>
     </row>
@@ -678,7 +689,7 @@
       <c r="A15" t="s">
         <v>16</v>
       </c>
-      <c r="B15" s="6" t="s">
+      <c r="B15" s="7" t="s">
         <v>17</v>
       </c>
     </row>
@@ -686,7 +697,7 @@
       <c r="A16" t="s">
         <v>18</v>
       </c>
-      <c r="B16" s="6" t="s">
+      <c r="B16" s="7" t="s">
         <v>19</v>
       </c>
     </row>
@@ -694,21 +705,21 @@
       <c r="A17" t="s">
         <v>20</v>
       </c>
-      <c r="B17" s="6" t="s">
+      <c r="B17" s="7" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A19" s="3" t="s">
+      <c r="A19" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="B19" s="4"/>
+      <c r="B19" s="5"/>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A20" s="5" t="s">
+      <c r="A20" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="B20" s="5" t="s">
+      <c r="B20" s="6" t="s">
         <v>11</v>
       </c>
     </row>
@@ -716,7 +727,7 @@
       <c r="A21" t="s">
         <v>23</v>
       </c>
-      <c r="B21" s="6" t="s">
+      <c r="B21" s="7" t="s">
         <v>24</v>
       </c>
     </row>
@@ -724,7 +735,7 @@
       <c r="A22" t="s">
         <v>25</v>
       </c>
-      <c r="B22" s="6" t="s">
+      <c r="B22" s="7" t="s">
         <v>26</v>
       </c>
     </row>
@@ -732,7 +743,7 @@
       <c r="A23" t="s">
         <v>27</v>
       </c>
-      <c r="B23" s="6" t="s">
+      <c r="B23" s="7" t="s">
         <v>19</v>
       </c>
     </row>
@@ -740,7 +751,7 @@
       <c r="A24" t="s">
         <v>28</v>
       </c>
-      <c r="B24" s="6" t="s">
+      <c r="B24" s="7" t="s">
         <v>29</v>
       </c>
     </row>
@@ -748,7 +759,7 @@
       <c r="A25" t="s">
         <v>30</v>
       </c>
-      <c r="B25" s="6" t="s">
+      <c r="B25" s="7" t="s">
         <v>31</v>
       </c>
     </row>
@@ -756,21 +767,21 @@
       <c r="A26" t="s">
         <v>32</v>
       </c>
-      <c r="B26" s="6" t="s">
+      <c r="B26" s="7" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A28" s="3" t="s">
+      <c r="A28" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="B28" s="4"/>
+      <c r="B28" s="5"/>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A29" s="5" t="s">
+      <c r="A29" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="B29" s="5" t="s">
+      <c r="B29" s="6" t="s">
         <v>35</v>
       </c>
     </row>
@@ -778,7 +789,7 @@
       <c r="A30" t="s">
         <v>36</v>
       </c>
-      <c r="B30" s="6" t="s">
+      <c r="B30" s="7" t="s">
         <v>21</v>
       </c>
     </row>
@@ -786,21 +797,21 @@
       <c r="A31" t="s">
         <v>37</v>
       </c>
-      <c r="B31" s="6" t="s">
+      <c r="B31" s="7" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A33" s="3" t="s">
+      <c r="A33" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="B33" s="4"/>
+      <c r="B33" s="5"/>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A34" s="5" t="s">
+      <c r="A34" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="B34" s="5" t="s">
+      <c r="B34" s="6" t="s">
         <v>40</v>
       </c>
     </row>
@@ -808,7 +819,7 @@
       <c r="A35" t="s">
         <v>41</v>
       </c>
-      <c r="B35" s="6" t="s">
+      <c r="B35" s="7" t="s">
         <v>21</v>
       </c>
     </row>
@@ -816,7 +827,7 @@
       <c r="A36" t="s">
         <v>42</v>
       </c>
-      <c r="B36" s="6" t="s">
+      <c r="B36" s="7" t="s">
         <v>29</v>
       </c>
     </row>
@@ -824,7 +835,7 @@
       <c r="A37" t="s">
         <v>43</v>
       </c>
-      <c r="B37" s="6" t="s">
+      <c r="B37" s="7" t="s">
         <v>44</v>
       </c>
     </row>
@@ -832,7 +843,7 @@
       <c r="A38" t="s">
         <v>45</v>
       </c>
-      <c r="B38" s="6" t="s">
+      <c r="B38" s="7" t="s">
         <v>21</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update KPI report exports to match on-screen layout and data display
Refactor KPI report exports to align PDF and Excel outputs with on-screen UI, including updated card layouts, date range formatting to DD.MM.YYYY, specific worker type listings, and conditional display of HGV-only metrics.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 0e10bf15-1a2d-43bc-934e-464c51d00f66
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: c6c486b9-c82f-490c-8028-513ac13fa6b3
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/9f621e76-a1cb-47c9-a804-6aa67d168f25/0e10bf15-1a2d-43bc-934e-464c51d00f66/HJE4Rfv
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/exports/kpi-report-sample.xlsx
+++ b/exports/kpi-report-sample.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="53">
   <si>
     <t>ShiftControl — KPI Report</t>
   </si>
@@ -25,19 +25,19 @@
     <t>Date range</t>
   </si>
   <si>
-    <t>19 Jul – 25 Jul 2026</t>
+    <t>01.07.2026 - 31.07.2026</t>
   </si>
   <si>
     <t>Worker type</t>
   </si>
   <si>
-    <t>HGV</t>
+    <t>HGV and Warehouse</t>
   </si>
   <si>
     <t>Report generated</t>
   </si>
   <si>
-    <t>22 July 2026, 08:45</t>
+    <t>22 July 2026, 09:57</t>
   </si>
   <si>
     <t>OPERATIONAL</t>
@@ -103,13 +103,13 @@
     <t>2</t>
   </si>
   <si>
-    <t>CPC failures (HGV only)</t>
+    <t>CPC failures</t>
   </si>
   <si>
     <t>0</t>
   </si>
   <si>
-    <t>Test failures (HGV only)</t>
+    <t>Test failures</t>
   </si>
   <si>
     <t>LEAVER REASONS (total 2)</t>
@@ -127,6 +127,21 @@
     <t>Travel Distance</t>
   </si>
   <si>
+    <t>Permanent Employment</t>
+  </si>
+  <si>
+    <t>Shift Pattern</t>
+  </si>
+  <si>
+    <t>Performance Issues</t>
+  </si>
+  <si>
+    <t>Attendance Issues</t>
+  </si>
+  <si>
+    <t>Other</t>
+  </si>
+  <si>
     <t>RETENTION BY LENGTH OF SERVICE (current snapshot)</t>
   </si>
   <si>
@@ -140,6 +155,12 @@
   </si>
   <si>
     <t>1–4 weeks</t>
+  </si>
+  <si>
+    <t>1–3 months</t>
+  </si>
+  <si>
+    <t>3–6 months</t>
   </si>
   <si>
     <t>6 months+</t>
@@ -610,7 +631,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A5:B38"/>
+  <dimension ref="A5:B45"/>
   <sheetFormatPr defaultRowHeight="16" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="44" customWidth="1"/>
@@ -801,18 +822,28 @@
         <v>21</v>
       </c>
     </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>38</v>
+      </c>
+      <c r="B32" s="7" t="s">
+        <v>31</v>
+      </c>
+    </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A33" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="B33" s="5"/>
+      <c r="A33" t="s">
+        <v>39</v>
+      </c>
+      <c r="B33" s="7" t="s">
+        <v>31</v>
+      </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A34" s="6" t="s">
-        <v>39</v>
-      </c>
-      <c r="B34" s="6" t="s">
+      <c r="A34" t="s">
         <v>40</v>
+      </c>
+      <c r="B34" s="7" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.25">
@@ -820,7 +851,7 @@
         <v>41</v>
       </c>
       <c r="B35" s="7" t="s">
-        <v>21</v>
+        <v>31</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.25">
@@ -828,22 +859,68 @@
         <v>42</v>
       </c>
       <c r="B36" s="7" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A38" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="B38" s="5"/>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A39" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="B39" s="6" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>46</v>
+      </c>
+      <c r="B40" s="7" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>47</v>
+      </c>
+      <c r="B41" s="7" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A37" t="s">
-        <v>43</v>
-      </c>
-      <c r="B37" s="7" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A38" t="s">
-        <v>45</v>
-      </c>
-      <c r="B38" s="7" t="s">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>48</v>
+      </c>
+      <c r="B42" s="7" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>49</v>
+      </c>
+      <c r="B43" s="7" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>50</v>
+      </c>
+      <c r="B44" s="7" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>52</v>
+      </c>
+      <c r="B45" s="7" t="s">
         <v>21</v>
       </c>
     </row>

</xml_diff>